<commit_message>
Modificar actividad: Diplomatura en Iniciación a la Programación y Análisis de Datos
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,11 +508,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46202</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -705,15 +707,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17 y 18/07/2026</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -723,7 +725,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -738,7 +740,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Jóvenes</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -755,22 +757,26 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
+          <t>CIC C/ Amancay y Canchas Calvo</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1381,7 +1387,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acto de entrega de certificados Programación </t>
+          <t xml:space="preserve">Entrega de certificados Programación </t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1668,6 +1674,73 @@
       </c>
       <c r="Q17" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sin especificar (Agosto 2026)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>31</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Entrega de certificados Programación</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SEEyA | UBA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Jóvenes y adultos</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modificar actividad: Incio Diplomatura Mediciones Nucleares
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -556,22 +556,26 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
+          <t>CIC C/ Amancay y Canchas Calvo</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Eliminar actividad fila 1
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,19 +580,19 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lanzamiento Programa Desafíos</t>
+          <t>Entrega de Diplomas y Cierre Nuclear</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> General Roca</t>
+          <t xml:space="preserve">San Carlos de Bariloche </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -603,7 +603,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizado</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>JUNIO</t>
+          <t>JULIO</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -644,41 +644,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46206</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Entrega de Diplomas y Cierre Nuclear</t>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">San Carlos de Bariloche </t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Finalizado</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INTERMEDIA</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -690,46 +696,50 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+          <t>CIC C/ Amancay y Canchas Calvo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>16 y 17 /07/2026</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>General Roca</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -761,32 +771,28 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Sin Ciudad</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>CIC C/ Amancay y Canchas Calvo</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Clase presencial</t>
-        </is>
-      </c>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16 y 17 /07/2026</t>
+          <t>17 y 18/07/2026</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -799,7 +805,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Roca</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -857,7 +863,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17 y 18/07/2026</t>
+          <t>20 y 21/07/2026</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -870,7 +876,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Roca</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -928,11 +934,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20 y 21/07/2026</t>
+          <t>30 y 31/07/2026</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -941,7 +947,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -961,7 +967,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t xml:space="preserve"> Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -999,11 +1005,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>30 y 31/07/2026</t>
+          <t>24 y 25/07/2026</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1012,7 +1018,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1032,7 +1038,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jóvenes y adultos</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1070,101 +1076,114 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24 y 25/07/2026</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Jornada de Integración para el Desarrollo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
+          <t xml:space="preserve">SEEyA | UBA </t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Clase presencial</t>
+          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Estudiantes/docentes/funcionarios/empresas</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>En curso</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>INTERMEDIA</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>JULIO</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEyA</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>SEEyA - Los Sauces y Los Arrayanes</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
+</t>
+        </is>
+      </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t xml:space="preserve">    3 y 4/07/2026</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jornada de Integración para el Desarrollo</t>
+          <t xml:space="preserve">Presencial Diplomatura Programación </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEEyA | UBA </t>
+          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
+          <t>Cursado Presencial</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1174,12 +1193,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Estudiantes/docentes/funcionarios/empresas</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INTERMEDIA</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1192,48 +1211,39 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria de EEyA</t>
-        </is>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Sin Ciudad</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>SEEyA - Los Sauces y Los Arrayanes</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
-</t>
-        </is>
-      </c>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3 y 4/07/2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presencial Diplomatura Programación </t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1243,12 +1253,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
+          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Cursado Presencial</t>
+          <t>17.30-Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1263,7 +1273,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>INTERMEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1276,7 +1286,11 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
           <t>Sin especificar</t>
@@ -1284,7 +1298,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1292,15 +1306,19 @@
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1308,22 +1326,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Entrega de certificados Programación</t>
+          <t xml:space="preserve">Entrega de certificados Programación </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
+          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>17.30-Entrega de certificados con autoridades</t>
+          <t>Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1353,7 +1371,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1363,7 +1381,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1377,36 +1395,36 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega de certificados Programación </t>
+          <t>Expo Universitaria</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
+          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Entrega de certificados con autoridades</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1416,7 +1434,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t>Estudiantes de nivel secundario y público en general</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1436,62 +1454,54 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
+          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Expo Universitaria</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Sierra Grande</t>
-        </is>
-      </c>
+          <t>Plenario del CIN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
-        </is>
-      </c>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1499,7 +1509,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Estudiantes de nivel secundario y público en general</t>
+          <t>Rectores de universidades de todo el país</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1507,63 +1517,55 @@
           <t>ALTA</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
+          <t xml:space="preserve">Gobernador </t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>San Carlos de Bariloche</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Plenario del CIN</t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UNRN</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1574,7 +1576,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Rectores de universidades de todo el país</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1586,41 +1588,41 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gobernador </t>
+          <t>Gobernador + Secretaria de EEyA</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>San Carlos de Bariloche</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>Sin especificar (Agosto 2026)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1630,7 +1632,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>SEEyA | UBA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1653,22 +1655,22 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA</t>
+          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1677,73 +1679,6 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Sin especificar (Agosto 2026)</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>31</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Entrega de certificados Programación</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>SEEyA | UBA</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>General Roca</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
-        </is>
-      </c>
-      <c r="Q18" t="n">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Eliminar actividad fila 2
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,7 +652,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16 y 17 /07/2026</t>
+          <t>17 y 18/07/2026</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Roca</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -723,7 +723,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17 y 18/07/2026</t>
+          <t>20 y 21/07/2026</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -736,7 +736,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Roca</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -794,11 +794,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20 y 21/07/2026</t>
+          <t>30 y 31/07/2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t xml:space="preserve"> Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -865,11 +865,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>30 y 31/07/2026</t>
+          <t>24 y 25/07/2026</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jóvenes y adultos</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -936,101 +936,114 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24 y 25/07/2026</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Jornada de Integración para el Desarrollo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
+          <t xml:space="preserve">SEEyA | UBA </t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Clase presencial</t>
+          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Estudiantes/docentes/funcionarios/empresas</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>En curso</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>INTERMEDIA</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>JULIO</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEyA</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>SEEyA - Los Sauces y Los Arrayanes</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
+</t>
+        </is>
+      </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t xml:space="preserve">    3 y 4/07/2026</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Jornada de Integración para el Desarrollo</t>
+          <t xml:space="preserve">Presencial Diplomatura Programación </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEEyA | UBA </t>
+          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
+          <t>Cursado Presencial</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1040,12 +1053,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Estudiantes/docentes/funcionarios/empresas</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INTERMEDIA</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1058,48 +1071,39 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria de EEyA</t>
-        </is>
-      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Sin Ciudad</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>SEEyA - Los Sauces y Los Arrayanes</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
-</t>
-        </is>
-      </c>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3 y 4/07/2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presencial Diplomatura Programación </t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1109,12 +1113,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
+          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Cursado Presencial</t>
+          <t>17.30-Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1129,7 +1133,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>INTERMEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1142,7 +1146,11 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>Sin especificar</t>
@@ -1150,7 +1158,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1158,15 +1166,19 @@
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1174,22 +1186,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Entrega de certificados Programación</t>
+          <t xml:space="preserve">Entrega de certificados Programación </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
+          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.30-Entrega de certificados con autoridades</t>
+          <t>Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1219,7 +1231,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1229,7 +1241,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1243,36 +1255,36 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega de certificados Programación </t>
+          <t>Expo Universitaria</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
+          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Entrega de certificados con autoridades</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1282,7 +1294,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t>Estudiantes de nivel secundario y público en general</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1302,62 +1314,54 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
+          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Expo Universitaria</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Sierra Grande</t>
-        </is>
-      </c>
+          <t>Plenario del CIN</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
-        </is>
-      </c>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1365,7 +1369,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Estudiantes de nivel secundario y público en general</t>
+          <t>Rectores de universidades de todo el país</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1373,63 +1377,55 @@
           <t>ALTA</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
+          <t xml:space="preserve">Gobernador </t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>San Carlos de Bariloche</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Plenario del CIN</t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>UNRN</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1440,7 +1436,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Rectores de universidades de todo el país</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1452,41 +1448,41 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gobernador </t>
+          <t>Gobernador + Secretaria de EEyA</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>San Carlos de Bariloche</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>Sin especificar (Agosto 2026)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1496,7 +1492,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>SEEyA | UBA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1519,22 +1515,22 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA</t>
+          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1543,73 +1539,6 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Sin especificar (Agosto 2026)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>31</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Entrega de certificados Programación</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>SEEyA | UBA</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>General Roca</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
-        </is>
-      </c>
-      <c r="Q16" t="n">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Eliminar actividad fila 0
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,28 +506,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Incio Diplomatura Mediciones Nucleares</t>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sal Carlos de Bariloche</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Instituto Balseiro</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>En curso</t>
@@ -535,7 +539,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -545,7 +549,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>JUNIO</t>
+          <t>JULIO</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
@@ -577,25 +581,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>17 y 18/07/2026</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>General Roca</t>
+          <t>Roca</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -627,32 +631,28 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Sin Ciudad</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>CIC C/ Amancay y Canchas Calvo</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Clase presencial</t>
-        </is>
-      </c>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17 y 18/07/2026</t>
+          <t>20 y 21/07/2026</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Roca</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -723,11 +723,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20 y 21/07/2026</t>
+          <t>30 y 31/07/2026</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t xml:space="preserve"> Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -794,11 +794,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30 y 31/07/2026</t>
+          <t>24 y 25/07/2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jóvenes y adultos</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -865,101 +865,114 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24 y 25/07/2026</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Presencial Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Jornada de Integración para el Desarrollo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Secretaría de Estado de Energía y Ambiente | Facultad de Ciencias Exactas de la UBA, Municipio</t>
+          <t xml:space="preserve">SEEyA | UBA </t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Clase presencial</t>
+          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Estudiantes/docentes/funcionarios/empresas</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>En curso</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>INTERMEDIA</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>JULIO</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEyA</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Cipolletti</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+          <t>SEEyA - Los Sauces y Los Arrayanes</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
+</t>
+        </is>
+      </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t xml:space="preserve">    3 y 4/07/2026</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Jornada de Integración para el Desarrollo</t>
+          <t xml:space="preserve">Presencial Diplomatura Programación </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEEyA | UBA </t>
+          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Jornada de 9 a 17hs exposición y presentación de trabajos</t>
+          <t>Cursado Presencial</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -969,12 +982,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Estudiantes/docentes/funcionarios/empresas</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INTERMEDIA</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -987,48 +1000,39 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria de EEyA</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Cipolletti</t>
+          <t>Sin Ciudad</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>SEEyA - Los Sauces y Los Arrayanes</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Espacio de encuentro e intercambio en el marco de la Diplomatura en Iniciación a la Programación y Análisis de Datos impulsada por la Secretaría de Energía y Ambiente de la provincia de Río Negro en convenio con la Facultad de Ciencias Naturales y Exactas de la UBA.
-</t>
-        </is>
-      </c>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3 y 4/07/2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presencial Diplomatura Programación </t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1038,12 +1042,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
+          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cursado Presencial</t>
+          <t>17.30-Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1058,7 +1062,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>INTERMEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1071,7 +1075,11 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>Sin especificar</t>
@@ -1079,7 +1087,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1087,15 +1095,19 @@
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1103,22 +1115,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Entrega de certificados Programación</t>
+          <t xml:space="preserve">Entrega de certificados Programación </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
+          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>17.30-Entrega de certificados con autoridades</t>
+          <t>Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1148,7 +1160,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1158,7 +1170,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1172,36 +1184,36 @@
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega de certificados Programación </t>
+          <t>Expo Universitaria</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
+          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Entrega de certificados con autoridades</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1211,7 +1223,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t>Estudiantes de nivel secundario y público en general</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1231,62 +1243,54 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
+          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Expo Universitaria</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Sierra Grande</t>
-        </is>
-      </c>
+          <t>Plenario del CIN</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
-        </is>
-      </c>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1294,7 +1298,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Estudiantes de nivel secundario y público en general</t>
+          <t>Rectores de universidades de todo el país</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1302,63 +1306,55 @@
           <t>ALTA</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
+          <t xml:space="preserve">Gobernador </t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>San Carlos de Bariloche</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Plenario del CIN</t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>UNRN</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1369,7 +1365,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Rectores de universidades de todo el país</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1381,41 +1377,41 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gobernador </t>
+          <t>Gobernador + Secretaria de EEyA</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>San Carlos de Bariloche</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>Sin especificar (Agosto 2026)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1425,7 +1421,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>SEEyA | UBA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1448,22 +1444,22 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA</t>
+          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1472,73 +1468,6 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Sin especificar (Agosto 2026)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>31</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Entrega de certificados Programación</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>SEEyA | UBA</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>General Roca</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
-        </is>
-      </c>
-      <c r="Q15" t="n">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir actividad: Plenario del CIN
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1473,6 +1473,73 @@
       </c>
       <c r="Q14" t="n">
         <v>36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>36</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Plenario del CIN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rectores </t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Gobernador</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>San Carlos de Bariloche</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Sin espeficificar</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadir actividad: Diplomatura en Iniciación a la Programación y Análisis de Datos
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1540,6 +1540,69 @@
       </c>
       <c r="Q15" t="n">
         <v>50</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>29</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SEEyA | UBA</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Jóvenes y adultos</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>INTERMEDIA</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>CET 33</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadir actividad: Diplomatura en Iniciación a la Programación y Analisis de Datos
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1607,6 +1607,69 @@
       </c>
       <c r="Q16" t="n">
         <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>30</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Diplomatura en Iniciación a la Programación y Analisis de Datos</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SEEyA | UBA | Municipio de Río Colorado</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Jóvenes y adultos</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>INTERMEDIA</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Río Colorado</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>CERC C/ H. Yrigoyen y Belgrano</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Clase presencial</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eliminar actividad fila 6
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -965,15 +965,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3 y 4/07/2026</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presencial Diplomatura Programación </t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Facultad de Exactas UBA/Secretaria de Energía/Municipios</t>
+          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cursado Presencial</t>
+          <t>17.30-Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>INTERMEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1016,7 +1016,11 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
           <t>Sin especificar</t>
@@ -1024,7 +1028,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Sin Ciudad</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1032,15 +1036,19 @@
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+        </is>
+      </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1048,22 +1056,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Entrega de certificados Programación</t>
+          <t xml:space="preserve">Entrega de certificados Programación </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Río Colorado</t>
+          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>17.30-Entrega de certificados con autoridades</t>
+          <t>Entrega de certificados con autoridades</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1093,7 +1101,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + Funcionarios</t>
+          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1103,7 +1111,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1117,36 +1125,36 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega de certificados Programación </t>
+          <t>Expo Universitaria</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
+          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Entrega de certificados con autoridades</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1156,7 +1164,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t>Estudiantes de nivel secundario y público en general</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1176,62 +1184,54 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEYA + fFuncionarios</t>
+          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Cinco Saltos</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Expo Universitaria</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Sierra Grande</t>
-        </is>
-      </c>
+          <t>Plenario del CIN</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEEyA | Ministerio de Educación y DDHH | Municipalidad de Sierra Grande | Fundación YPF</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
-        </is>
-      </c>
+          <t>UNRN</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Estudiantes de nivel secundario y público en general</t>
+          <t>Rectores de universidades de todo el país</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1247,63 +1247,55 @@
           <t>ALTA</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA + Ministra de Educación + Funcionarios</t>
+          <t xml:space="preserve">Gobernador </t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>San Carlos de Bariloche</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Feria y exposiciones sobre carreras universitarios y formación terciaria</t>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Plenario del CIN</t>
+          <t>Entrega de certificados Programación</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>UNRN</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1314,7 +1306,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Rectores de universidades de todo el país</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1326,41 +1318,41 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gobernador </t>
+          <t>Gobernador + Secretaria de EEyA</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>San Carlos de Bariloche</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Gimnasio Vuta Mahuida</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>Sin especificar (Agosto 2026)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1370,7 +1362,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>SEEyA | UBA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1393,22 +1385,22 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria de EEyA</t>
+          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Gimnasio Vuta Mahuida</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1417,27 +1409,27 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sin especificar (Agosto 2026)</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Entrega de certificados Programación</t>
+          <t>Plenario del CIN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEEyA | UBA</t>
+          <t>UNRN</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1448,7 +1440,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Jóvenes y adultos</t>
+          <t>Rectores de universidades de todo el país</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1460,7 +1452,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Gobernador + Secretaria EEyA + Funcionarios</t>
+          <t>Gobernador</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1470,114 +1462,110 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>General Roca</t>
+          <t>San Carlos de Bariloche</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Sin espeficificar</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Acto de entrega de certificados de la Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Plenario del CIN</t>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>UNRN</t>
+          <t>SEEyA | UBA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Rectores de universidades de todo el país</t>
+          <t>Jóvenes y adultos</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INTERMEDIA</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Gobernador</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>San Carlos de Bariloche</t>
+          <t>General Roca</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Sin espeficificar</t>
+          <t>CET 33</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+          <t>Clase presencial</t>
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
+          <t>Diplomatura en Iniciación a la Programación y Analisis de Datos</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEEyA | UBA</t>
+          <t>SEEyA | UBA | Municipio de Río Colorado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1595,17 +1583,17 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>General Roca</t>
+          <t>Río Colorado</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>CET 33</t>
+          <t>CERC C/ H. Yrigoyen y Belgrano</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1614,33 +1602,33 @@
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Diplomatura en Iniciación a la Programación y Analisis de Datos</t>
+          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipio de Río Colorado</t>
+          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1658,17 +1646,17 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Río Colorado</t>
+          <t>Sierra Grande</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>CERC C/ H. Yrigoyen y Belgrano</t>
+          <t>CIC C/ Amancay y Canchas Calvo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1677,17 +1665,17 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1697,7 +1685,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEEyA | UBA | Municipalidad de Sierra Grande</t>
+          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1726,12 +1714,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Sierra Grande</t>
+          <t>Cinco Saltos</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>CIC C/ Amancay y Canchas Calvo</t>
+          <t>Escuela Primaria N° 291 C/ Pedro Ramos 849</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1740,69 +1728,6 @@
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>30</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Diplomatura en Iniciación a la Programación y Análisis de Datos</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SEEyA | UBA | Municipalidad de Cinco Saltos</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Jóvenes y adultos</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>INTERMEDIA</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Cinco Saltos</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Escuela Primaria N° 291 C/ Pedro Ramos 849</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Clase presencial</t>
-        </is>
-      </c>
-      <c r="Q19" t="n">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir actividad: Lanzamiento Dot conecta
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1731,6 +1731,57 @@
         <v>20</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>34</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lanzamiento Dot conecta</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>INTERMEDIA</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Diario Rio Negro</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: reunión en FADECS
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1782,6 +1782,61 @@
         <v>50</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>33</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>reunión en FADECS</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>FADECS</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasantias y otras articulaciones </t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Invitación a 3º expo vocacional
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1746,14 +1746,22 @@
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>INTERMEDIA</t>
@@ -1797,14 +1805,22 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -1837,6 +1853,57 @@
         <v>50</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>32</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invitación a 3º expo vocacional </t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Catriel</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>SUM Municipal</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Invitación 3º Expo vocacional
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1904,6 +1904,57 @@
         <v>50</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>32</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invitación 3º Expo vocacional </t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Catriel</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>SUM Municipal</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Encuentro virtual del Programa para el Desarrollo Productivo y Financiero de Mujeres
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1868,14 +1868,22 @@
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>BAJA</t>
@@ -1919,14 +1927,22 @@
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>BAJA</t>
@@ -1955,6 +1971,62 @@
         <v>50</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>32</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Encuentro virtual del Programa para el Desarrollo Productivo y Financiero de Mujeres</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Cipolleti</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>encuentro virtual para repasar el
+Estado de situación del Programa, novedades importantes: el lanzamiento de una Capacitación, nuevas herramientas financieras disponibles, y avances de la Red Federal de Mujeres para el Desarrollo.</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modificar actividad: Invitación 3º Expo vocacional
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -1986,14 +1986,22 @@
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>ALTA</t>

</xml_diff>

<commit_message>
Modificar actividad: 3º Expo Vocacional
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -1864,13 +1864,13 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invitación a 3º expo vocacional </t>
+          <t xml:space="preserve">3º Expo Vocacional </t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1907,7 +1907,11 @@
           <t>SUM Municipal</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Expo Vocacional</t>
+        </is>
+      </c>
       <c r="Q21" t="n">
         <v>50</v>
       </c>

</xml_diff>

<commit_message>
Eliminar actividad fila 19
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1856,7 +1856,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1864,13 +1864,13 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">3º Expo Vocacional </t>
+          <t xml:space="preserve">Invitación 3º Expo vocacional </t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1907,11 +1907,7 @@
           <t>SUM Municipal</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Expo Vocacional</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
         <v>50</v>
       </c>
@@ -1927,7 +1923,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invitación 3º Expo vocacional </t>
+          <t>Encuentro virtual del Programa para el Desarrollo Productivo y Financiero de Mujeres</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1949,7 +1945,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BAJA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1957,85 +1953,26 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Catriel</t>
+          <t>Cipolleti</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>SUM Municipal</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>32</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Encuentro virtual del Programa para el Desarrollo Productivo y Financiero de Mujeres</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Cipolleti</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>encuentro virtual para repasar el
 Estado de situación del Programa, novedades importantes: el lanzamiento de una Capacitación, nuevas herramientas financieras disponibles, y avances de la Red Federal de Mujeres para el Desarrollo.</t>
         </is>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q22" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir actividad: Expo Vocacional
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1917,6 +1917,65 @@
         <v>50</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>32</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Expo Vocacional</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Catriel</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>SUM Municipal Eldo Carro</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Evento para que los jóvenes conozcan la oferta académica de universidades, institutos y centros de educación superior, dialogar con referentes de cada institución y recibir orientación.</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Eliminar actividad fila 18
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1793,34 +1793,26 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>reunión en FADECS</t>
+          <t>Expo Vocacional</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -1828,87 +1820,32 @@
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>General Roca</t>
+          <t>Catriel</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>FADECS</t>
+          <t>SUM Municipal Eldo Carro</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pasantias y otras articulaciones </t>
+          <t>Evento para que los jóvenes conozcan la oferta académica de universidades, institutos y centros de educación superior, dialogar con referentes de cada institución y recibir orientación.</t>
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>32</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Expo Vocacional</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Catriel</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>SUM Municipal Eldo Carro</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Evento para que los jóvenes conozcan la oferta académica de universidades, institutos y centros de educación superior, dialogar con referentes de cada institución y recibir orientación.</t>
-        </is>
-      </c>
-      <c r="Q21" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modificar actividad: Jornada de Integración para el Desarrollo
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -881,11 +881,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Modificar actividad: Entrega de certificados Programación
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -965,11 +965,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Sin especificar (A coordinar)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">

</xml_diff>

<commit_message>
Modificar actividad: Plenario del CIN
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -1927,7 +1927,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1978,7 +1978,11 @@
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>El fin será contribuir con la elaboración de agendas institucionales y de política pública para el fortalecimiento de una educación superior democrática, federal y socialmente comprometida.</t>
+        </is>
+      </c>
       <c r="Q22" t="n">
         <v>50</v>
       </c>

</xml_diff>

<commit_message>
Añadir actividad: Jornada CFI - Gestión para el Desarrollo
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2058,6 +2058,65 @@
         <v>50</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>35</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Jornada CFI - Gestión para el Desarrollo</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CFI | SEEyA</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Jóvenes</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Alto Valle</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Jornada de integración y paneles provinciales compuestas por visitas a sitios estratégicos para el desarrollo de la provincia, encuentros con funcionarias/os y referentes locales y actividades de integración grupal con los participantes de la formación Gestión para el Desarrollo.</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: CFI - Jornada de Integración
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2117,6 +2117,65 @@
         <v>25</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>35</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CFI - Jornada de Integración</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CFI | SEEyE</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Jóvenes</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Alto Valle</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Jornada de integración y paneles provinciales compuestas por visitas a sitios estratégicos para el desarrollo de la provincia, encuentros con funcionarias/os y referentes locales y actividades de integración grupal con los participantes de la formación Gestión para el Desarrollo.</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: I Foro de la Juventud Rionegrina
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2042,6 +2042,69 @@
         <v>25</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>33</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>I Foro de la Juventud Rionegrina</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Jóvenes</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Cipolletti</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Escuela Manuel Belgrano | CCC</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primer Foro de la Juventud Rionegrina que reúne a jóvenes de toda la provincia para debatir, proponer y pensar la provincia. </t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>